<commit_message>
fix: update template and skill to match Chinese 发票 fields
Mandatory fields: 发票号码, 开票日期, 发票类型, 购买方名称, 购买方税号,
销售方名称, 销售方税号, 服务项目名称, 税率, 金额, 税额, 价税合计

Template: 15 columns (A-O), blue header, example row in gray.
Extraction prompt: Chinese field names with English translations.
Reply format: Chinese table format.
</commit_message>
<xml_diff>
--- a/.opencode/skills/invoice-processing/template.xlsx
+++ b/.opencode/skills/invoice-processing/template.xlsx
@@ -437,23 +437,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -469,60 +470,65 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>发票日期</t>
+          <t>开票日期</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>供应商/卖方</t>
+          <t>发票类型</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>商品/服务描述</t>
+          <t>购买方名称</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>金额(不含税)</t>
+          <t>购买方税号</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>销售方名称</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>销售方税号</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>服务项目名称</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>税率</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>金额</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>税额</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>价税合计</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>发票类型</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>付款状态</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>付款日期</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>文件名</t>
         </is>
@@ -544,45 +550,54 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>示例供应商</t>
+          <t>增值税普通发票</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>办公用品</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>100</v>
+          <t>示例购买方</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>91110000XXXXXXXX</t>
+        </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>13%</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="I2" s="2" t="n">
-        <v>113</v>
+          <t>示例销售方</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>91110000YYYYYYYY</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>信息技术服务</t>
+        </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>增值税普通发票</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>未付款</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr">
+          <t>6%</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>1060</v>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>示例数据，请删除</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>invoice_001.pdf</t>
         </is>

</xml_diff>